<commit_message>
Actualización Excel con los pines y su asignación al STM32F103C8T6
</commit_message>
<xml_diff>
--- a/analisis_hardware_midagi.xlsx
+++ b/analisis_hardware_midagi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pruebacorreoescuelaingeduco-my.sharepoint.com/personal/giovanny_torres_mail_escuelaing_edu_co/Documents/2026-1/MPEI-1/Acceso a GitHub/MIDAGI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pruebacorreoescuelaingeduco-my.sharepoint.com/personal/miguel_reina-c_mail_escuelaing_edu_co/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7542BE2B-E4EE-49C9-AF8F-F6A96716B66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F376FCC5-F0FF-4788-A4BD-A5A0BF4743F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="1" activeTab="1" xr2:uid="{32F234FD-9D53-4994-8ACD-9A380420451B}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="2" activeTab="2" xr2:uid="{32F234FD-9D53-4994-8ACD-9A380420451B}"/>
   </bookViews>
   <sheets>
     <sheet name="HARDWARE" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,82 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="299">
+  <si>
+    <t>PROYECTO MIDAGI</t>
+  </si>
+  <si>
+    <t>CANTIDAD</t>
+  </si>
+  <si>
+    <t>MATERIAL</t>
+  </si>
+  <si>
+    <t>PRECIO UN</t>
+  </si>
+  <si>
+    <t>PRECIO TOTAL</t>
+  </si>
+  <si>
+    <t>STM32F103</t>
+  </si>
+  <si>
+    <t>ESP8266 Modulo WI-FI</t>
+  </si>
+  <si>
+    <t>BATERIA 7.5V</t>
+  </si>
+  <si>
+    <t>SENSOR INFRARROJO IRS01A</t>
+  </si>
+  <si>
+    <t>FALTAN 2</t>
+  </si>
+  <si>
+    <t>SENSOR SHARP</t>
+  </si>
+  <si>
+    <t>INVESTIGAR FUNCIONAMIENTO</t>
+  </si>
+  <si>
+    <t>SENSOR DE IMPACTO PARA DETENCIÓN DE GOLPES KY031</t>
+  </si>
+  <si>
+    <t>PUENTE H TB6612FNG</t>
+  </si>
+  <si>
+    <t>CIRCUITO IMPRESO</t>
+  </si>
+  <si>
+    <t>SENSOR ULTRASONICO HC-SR04</t>
+  </si>
+  <si>
+    <t>CHASIS SUMO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUEDAS </t>
+  </si>
+  <si>
+    <t>MOTORES</t>
+  </si>
+  <si>
+    <t>SERVOMOTOR</t>
+  </si>
+  <si>
+    <t>FALTA 1</t>
+  </si>
+  <si>
+    <t>PANTALLA OLED</t>
+  </si>
+  <si>
+    <t>LED RGB</t>
+  </si>
+  <si>
+    <t>BUZZER</t>
+  </si>
+  <si>
+    <t>RUEDA LOCA</t>
+  </si>
   <si>
     <t>COMPONENTE</t>
   </si>
@@ -131,9 +206,6 @@
   </si>
   <si>
     <t>No, pero configurar BAUD RATE, NOMBRE, Modo AT</t>
-  </si>
-  <si>
-    <t>LED RGB</t>
   </si>
   <si>
     <t>Mezcla RGB para formar colores</t>
@@ -233,9 +305,6 @@
   </si>
   <si>
     <t>Se programa con la librería ESP8266WiFi.h en el IDE de Arduino, a menudo usando comandos AT</t>
-  </si>
-  <si>
-    <t>SENSOR SHARP</t>
   </si>
   <si>
     <t xml:space="preserve">VCC
@@ -378,7 +447,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Conectar los dos cables del motor a las terminales </t>
@@ -389,7 +457,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>OUT1</t>
@@ -399,7 +466,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> y </t>
@@ -410,7 +476,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>OUT2</t>
@@ -420,7 +485,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -453,7 +517,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Conectar los dos cables del motor a las terminales </t>
@@ -464,7 +527,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>OUT3</t>
@@ -474,7 +536,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> y </t>
@@ -485,7 +546,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>OUT4</t>
@@ -495,7 +555,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -566,9 +625,6 @@
   </si>
   <si>
     <t>Aca se usara un transistor NPN 2N2222</t>
-  </si>
-  <si>
-    <t>BUZZER</t>
   </si>
   <si>
     <t>(+)</t>
@@ -583,7 +639,6 @@
         <sz val="11"/>
         <color rgb="FF1F1F1F"/>
         <rFont val="Aptos Display"/>
-        <family val="2"/>
         <scheme val="major"/>
       </rPr>
       <t xml:space="preserve">Colector </t>
@@ -593,7 +648,6 @@
         <sz val="11"/>
         <color rgb="FF1F1F1F"/>
         <rFont val="Aptos Display"/>
-        <family val="2"/>
         <scheme val="major"/>
       </rPr>
       <t>de 2N2222 al (-)</t>
@@ -606,7 +660,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Emisor</t>
@@ -616,7 +669,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> al GND</t>
@@ -628,7 +680,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">La </t>
@@ -639,7 +690,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>BASE</t>
@@ -649,7 +699,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> al pin </t>
@@ -660,7 +709,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>PB2 con una resistencia de 1k</t>
@@ -754,9 +802,6 @@
     <t>El azul también funciona a unos 3V.</t>
   </si>
   <si>
-    <t>PANTALLA OLED</t>
-  </si>
-  <si>
     <t>SCL</t>
   </si>
   <si>
@@ -772,251 +817,338 @@
     <t>PB7</t>
   </si>
   <si>
-    <t>SENSOR</t>
+    <t>SENSOR / MÓDULO</t>
+  </si>
+  <si>
+    <t>Voltaje</t>
+  </si>
+  <si>
+    <t>IN or OUT</t>
+  </si>
+  <si>
+    <t>Tipo de Señal</t>
+  </si>
+  <si>
+    <t>ASIGNACIÓN</t>
   </si>
   <si>
     <t>PIN_STM32</t>
   </si>
   <si>
-    <t>ASIGNACIÓN</t>
+    <t>Tipo_Pin</t>
+  </si>
+  <si>
+    <t>MONITOREO CORRIENTE</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>Analog</t>
+  </si>
+  <si>
+    <t>SYS_CURR</t>
+  </si>
+  <si>
+    <t>ADC1_IN0</t>
+  </si>
+  <si>
+    <t>STM32F103C8T6</t>
+  </si>
+  <si>
+    <t>0A41SK SHARP 1</t>
+  </si>
+  <si>
+    <t>SH1_SIG</t>
+  </si>
+  <si>
+    <t>PA4</t>
+  </si>
+  <si>
+    <t>ADC1_IN4</t>
+  </si>
+  <si>
+    <t>0A41SK SHARP 2</t>
+  </si>
+  <si>
+    <t>SH2_SIG</t>
+  </si>
+  <si>
+    <t>PA5</t>
+  </si>
+  <si>
+    <t>ADC1_IN5</t>
+  </si>
+  <si>
+    <t>0A41SK SHARP 3</t>
+  </si>
+  <si>
+    <t>SH3_SIG</t>
+  </si>
+  <si>
+    <t>PB0</t>
+  </si>
+  <si>
+    <t>ADC1_IN8</t>
+  </si>
+  <si>
+    <t>MONITOREO BATERIA</t>
+  </si>
+  <si>
+    <t>BAT_VOL</t>
+  </si>
+  <si>
+    <t>PB1</t>
+  </si>
+  <si>
+    <t>ADC1_IN9</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>BOTON MODO</t>
+  </si>
+  <si>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>BTN_MODE</t>
+  </si>
+  <si>
+    <t>PB2</t>
+  </si>
+  <si>
+    <t>GPIO_Input</t>
+  </si>
+  <si>
+    <t>HC-SR04 ULTRASONIDO</t>
   </si>
   <si>
     <t>US_ECHO</t>
   </si>
   <si>
+    <t>PA12</t>
+  </si>
+  <si>
+    <t>IRS01A INFRAROJO 1</t>
+  </si>
+  <si>
+    <t>IR1_SIG</t>
+  </si>
+  <si>
+    <t>PB5</t>
+  </si>
+  <si>
+    <t>IRS01A INFRAROJO 2</t>
+  </si>
+  <si>
+    <t>IR2_SIG</t>
+  </si>
+  <si>
+    <t>PB4</t>
+  </si>
+  <si>
+    <t>IRS01A INFRAROJO 3</t>
+  </si>
+  <si>
+    <t>IR3_SIG</t>
+  </si>
+  <si>
+    <t>IRS01A INFRAROJO 4</t>
+  </si>
+  <si>
+    <t>IR4_SIG</t>
+  </si>
+  <si>
+    <t>KY-031 IMPACTO 1</t>
+  </si>
+  <si>
+    <t>KY1_SIG</t>
+  </si>
+  <si>
+    <t>PB3</t>
+  </si>
+  <si>
+    <t>KY-031 IMPACTO 2</t>
+  </si>
+  <si>
+    <t>KY2_SIG</t>
+  </si>
+  <si>
+    <t>PC13</t>
+  </si>
+  <si>
+    <t>KY-031 IMPACTO 3</t>
+  </si>
+  <si>
+    <t>KY3_SIG</t>
+  </si>
+  <si>
+    <t>PC14</t>
+  </si>
+  <si>
+    <t>BUZZ_SIG</t>
+  </si>
+  <si>
+    <t>PC15</t>
+  </si>
+  <si>
+    <t>GPIO_Output</t>
+  </si>
+  <si>
     <t>US_TRIG</t>
   </si>
   <si>
-    <t>SHARP_1</t>
-  </si>
-  <si>
-    <t>PA4</t>
-  </si>
-  <si>
-    <t>SH1_SIG</t>
-  </si>
-  <si>
-    <t>SHARP_2</t>
-  </si>
-  <si>
-    <t>PA5</t>
-  </si>
-  <si>
-    <t>SHARP_3</t>
-  </si>
-  <si>
-    <t>PB0</t>
-  </si>
-  <si>
-    <t>SERVO_1</t>
+    <t>PA15</t>
+  </si>
+  <si>
+    <t>PH_IN1</t>
+  </si>
+  <si>
+    <t>PH_IN2</t>
+  </si>
+  <si>
+    <t>PH_IN3</t>
+  </si>
+  <si>
+    <t>PH_IN4</t>
+  </si>
+  <si>
+    <t>JMD0.96D-1 OLED</t>
+  </si>
+  <si>
+    <t>Digital (I2C)</t>
+  </si>
+  <si>
+    <t>OLED_SCL</t>
+  </si>
+  <si>
+    <t>I2C1_SCL</t>
+  </si>
+  <si>
+    <t>IN/OUT</t>
+  </si>
+  <si>
+    <t>OLED_SDA</t>
+  </si>
+  <si>
+    <t>I2C1_SDA</t>
+  </si>
+  <si>
+    <t>SG90 SERVO 1</t>
+  </si>
+  <si>
+    <t>Digital (PWM)</t>
+  </si>
+  <si>
+    <t>SER1_SIG</t>
   </si>
   <si>
     <t>PA8</t>
   </si>
   <si>
-    <t>SER1_SIG</t>
-  </si>
-  <si>
-    <t>SERVO_2</t>
+    <t>TIM1_CH1</t>
   </si>
   <si>
     <t>SER2_SIG</t>
   </si>
   <si>
+    <t>PA11</t>
+  </si>
+  <si>
+    <t>TIM1_CH4</t>
+  </si>
+  <si>
+    <t>LED RGB (Rojo)</t>
+  </si>
+  <si>
+    <t>REG_RED</t>
+  </si>
+  <si>
+    <t>TIM2_CH2</t>
+  </si>
+  <si>
+    <t>LED RGB (Verde)</t>
+  </si>
+  <si>
+    <t>REG_GREEN</t>
+  </si>
+  <si>
+    <t>TIM2_CH3</t>
+  </si>
+  <si>
+    <t>LED RGB (Azul)</t>
+  </si>
+  <si>
+    <t>REG_BLUE</t>
+  </si>
+  <si>
+    <t>TIM2_CH4</t>
+  </si>
+  <si>
     <t>PH_ENA</t>
   </si>
   <si>
-    <t>PH_IN1</t>
-  </si>
-  <si>
-    <t>PH_IN2</t>
+    <t>PB8</t>
+  </si>
+  <si>
+    <t>TIM4_CH3</t>
   </si>
   <si>
     <t>PH_ENB</t>
   </si>
   <si>
-    <t>PH_IN3</t>
-  </si>
-  <si>
-    <t>PH_IN4</t>
-  </si>
-  <si>
-    <t>INFRAROJO 1 IRS01A</t>
-  </si>
-  <si>
-    <t>PB3</t>
-  </si>
-  <si>
-    <t>IR1_SIG</t>
-  </si>
-  <si>
-    <t>INFRAROJO 2 IRS01A</t>
-  </si>
-  <si>
-    <t>PB4</t>
-  </si>
-  <si>
-    <t>IR2_SIG</t>
-  </si>
-  <si>
-    <t>INFRAROJO 3 IRS01A</t>
-  </si>
-  <si>
-    <t>PB8</t>
-  </si>
-  <si>
-    <t>IR3_SIG</t>
-  </si>
-  <si>
-    <t>INFRAROJO 4 IRS01A</t>
-  </si>
-  <si>
     <t>PB9</t>
   </si>
   <si>
-    <t>IR4_SIG</t>
-  </si>
-  <si>
-    <t>IMPACTO 1</t>
-  </si>
-  <si>
-    <t>PA15</t>
-  </si>
-  <si>
-    <t>KY1_SIG</t>
-  </si>
-  <si>
-    <t>IMPACTO 2</t>
+    <t>TIM4_CH4</t>
+  </si>
+  <si>
+    <t>HC-05 BLUETOOTH</t>
+  </si>
+  <si>
+    <t>Digital (UART)</t>
+  </si>
+  <si>
+    <t>BT_TX</t>
+  </si>
+  <si>
+    <t>USART1_RX</t>
+  </si>
+  <si>
+    <t>BT_RX</t>
+  </si>
+  <si>
+    <t>USART1_TX</t>
+  </si>
+  <si>
+    <t>ESP8266 WI-FI</t>
+  </si>
+  <si>
+    <t>WIFI_TX</t>
+  </si>
+  <si>
+    <t>PB11</t>
+  </si>
+  <si>
+    <t>USART3_RX</t>
+  </si>
+  <si>
+    <t>WIFI_RX</t>
   </si>
   <si>
     <t>PB10</t>
   </si>
   <si>
-    <t>KY2_SIG</t>
-  </si>
-  <si>
-    <t>IMPACTO 3</t>
-  </si>
-  <si>
-    <t>PB11</t>
-  </si>
-  <si>
-    <t>KY3_SIG</t>
-  </si>
-  <si>
-    <t>PB2</t>
-  </si>
-  <si>
-    <t>BUZZ_SIG</t>
-  </si>
-  <si>
-    <t>BT_TX</t>
-  </si>
-  <si>
-    <t>BT_RX</t>
-  </si>
-  <si>
-    <t>WI-FI</t>
-  </si>
-  <si>
-    <t>WIFI_TX</t>
-  </si>
-  <si>
-    <t>WIFI_RX</t>
-  </si>
-  <si>
-    <t>PC13</t>
-  </si>
-  <si>
-    <t>REG_RED</t>
-  </si>
-  <si>
-    <t>PC14</t>
-  </si>
-  <si>
-    <t>REG_GREEN</t>
-  </si>
-  <si>
-    <t>PC15</t>
-  </si>
-  <si>
-    <t>REG_BLUE</t>
-  </si>
-  <si>
-    <t>OLED_SCL</t>
-  </si>
-  <si>
-    <t>OLED_SDA</t>
-  </si>
-  <si>
-    <t>PROYECTO MIDAGI</t>
-  </si>
-  <si>
-    <t>CANTIDAD</t>
-  </si>
-  <si>
-    <t>MATERIAL</t>
-  </si>
-  <si>
-    <t>PRECIO UN</t>
-  </si>
-  <si>
-    <t>PRECIO TOTAL</t>
-  </si>
-  <si>
-    <t>STM32F103</t>
-  </si>
-  <si>
-    <t>ESP8266 Modulo WI-FI</t>
-  </si>
-  <si>
-    <t>BATERIA 7.5V</t>
-  </si>
-  <si>
-    <t>SENSOR INFRARROJO IRS01A</t>
-  </si>
-  <si>
-    <t>FALTAN 2</t>
-  </si>
-  <si>
-    <t>INVESTIGAR FUNCIONAMIENTO</t>
-  </si>
-  <si>
-    <t>SENSOR DE IMPACTO PARA DETENCIÓN DE GOLPES KY031</t>
-  </si>
-  <si>
-    <t>PUENTE H TB6612FNG</t>
-  </si>
-  <si>
-    <t>CIRCUITO IMPRESO</t>
-  </si>
-  <si>
-    <t>SENSOR ULTRASONICO HC-SR04</t>
-  </si>
-  <si>
-    <t>CHASIS SUMO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUEDAS </t>
-  </si>
-  <si>
-    <t>MOTORES</t>
-  </si>
-  <si>
-    <t>SERVOMOTOR</t>
-  </si>
-  <si>
-    <t>FALTA 1</t>
-  </si>
-  <si>
-    <t>RUEDA LOCA</t>
+    <t>USART3_TX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1037,14 +1169,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
@@ -1052,21 +1182,18 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF1F1F1F"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
@@ -1074,7 +1201,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
@@ -1082,21 +1208,18 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1110,14 +1233,24 @@
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Aptos Display"/>
-      <family val="2"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1440,7 +1573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1599,114 +1732,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1717,11 +1742,220 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1737,6 +1971,25 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E77FFE65-CAAB-48E9-B266-0FD9F8368BAB}" name="Tabla2" displayName="Tabla2" ref="A1:G34" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G34" xr:uid="{E77FFE65-CAAB-48E9-B266-0FD9F8368BAB}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G34">
+    <sortCondition ref="G1:G34"/>
+  </sortState>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{C9F7B643-C81A-4198-9B7D-BD7ABC74C34E}" name="SENSOR / MÓDULO" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B8B7038D-52C4-46B9-B98F-1B0AE09A1790}" name="Voltaje" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{3AD7EE40-942D-433F-9231-4CF71E618CB0}" name="IN or OUT" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{7586CE55-784F-4B82-81CF-00B4EF017135}" name="Tipo de Señal" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{A35757F3-8C96-4EC2-8E24-D99CA53F5FFE}" name="ASIGNACIÓN" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{F1367258-CB79-4984-908C-826730881A57}" name="PIN_STM32" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{1685FCBE-2C38-4793-A84A-B08DAE2637DD}" name="Tipo_Pin" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2057,215 +2310,215 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C61E87F0-6530-4D34-A6C8-ECF2EC7DB359}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.1015625" customWidth="1"/>
-    <col min="2" max="2" width="48.7890625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.89453125" customWidth="1"/>
-    <col min="4" max="4" width="23.3125" customWidth="1"/>
-    <col min="5" max="5" width="26.89453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="90" t="s">
-        <v>228</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="91" t="s">
-        <v>229</v>
-      </c>
-      <c r="B2" s="91" t="s">
-        <v>230</v>
-      </c>
-      <c r="C2" s="91" t="s">
-        <v>231</v>
-      </c>
-      <c r="D2" s="91" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="92">
+    <row r="1" spans="1:5">
+      <c r="A1" s="65" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="92" t="s">
-        <v>233</v>
-      </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="92">
+      <c r="B2" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="55" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="56">
         <v>1</v>
       </c>
-      <c r="B4" s="92" t="s">
-        <v>234</v>
-      </c>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="92">
+      <c r="B3" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="56">
         <v>1</v>
       </c>
-      <c r="B5" s="92" t="s">
-        <v>235</v>
-      </c>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="92">
+      <c r="B4" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="56">
+        <v>1</v>
+      </c>
+      <c r="B5" s="56" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="56">
         <v>4</v>
       </c>
-      <c r="B6" s="92" t="s">
-        <v>236</v>
-      </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
+      <c r="B6" s="56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
       <c r="E6" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="92">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="56">
         <v>6</v>
       </c>
-      <c r="B7" s="92" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="92"/>
-      <c r="D7" s="92"/>
-      <c r="E7" s="93" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="92">
+      <c r="B7" s="56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="56"/>
+      <c r="D7" s="56"/>
+      <c r="E7" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="56">
         <v>4</v>
       </c>
-      <c r="B8" s="92" t="s">
-        <v>239</v>
-      </c>
-      <c r="C8" s="92"/>
-      <c r="D8" s="92"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="92">
+      <c r="B8" s="56" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="56">
         <v>1</v>
       </c>
-      <c r="B9" s="92" t="s">
-        <v>240</v>
-      </c>
-      <c r="C9" s="92"/>
-      <c r="D9" s="92"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="94">
+      <c r="B9" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="58">
         <v>1</v>
       </c>
-      <c r="B10" s="94" t="s">
-        <v>241</v>
-      </c>
-      <c r="C10" s="94"/>
-      <c r="D10" s="94"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="92">
+      <c r="B10" s="58" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="56">
         <v>1</v>
       </c>
-      <c r="B11" s="95" t="s">
-        <v>242</v>
-      </c>
-      <c r="C11" s="92"/>
-      <c r="D11" s="92"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="94">
+      <c r="B11" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="56"/>
+      <c r="D11" s="56"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="58">
         <v>1</v>
       </c>
-      <c r="B12" s="94" t="s">
-        <v>243</v>
-      </c>
-      <c r="C12" s="94"/>
-      <c r="D12" s="94"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="92">
+      <c r="B12" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="56">
         <v>2</v>
       </c>
-      <c r="B13" s="92" t="s">
-        <v>244</v>
-      </c>
-      <c r="C13" s="92"/>
-      <c r="D13" s="92"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="92">
+      <c r="B13" s="56" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="56"/>
+      <c r="D13" s="56"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="56">
         <v>2</v>
       </c>
-      <c r="B14" s="92" t="s">
-        <v>245</v>
-      </c>
-      <c r="C14" s="92"/>
-      <c r="D14" s="92"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="92">
+      <c r="B14" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="56">
         <v>2</v>
       </c>
-      <c r="B15" s="92" t="s">
-        <v>246</v>
-      </c>
-      <c r="C15" s="92"/>
-      <c r="D15" s="92"/>
+      <c r="B15" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
       <c r="E15" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="92">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="56">
         <v>1</v>
       </c>
-      <c r="B16" s="92" t="s">
-        <v>163</v>
-      </c>
-      <c r="C16" s="92"/>
-      <c r="D16" s="92"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="92">
+      <c r="B16" s="56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="56">
         <v>1</v>
       </c>
-      <c r="B17" s="92" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="92"/>
-      <c r="D17" s="92"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="92">
+      <c r="B17" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="56">
         <v>1</v>
       </c>
-      <c r="B18" s="92" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="92"/>
-      <c r="D18" s="92"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="96">
+      <c r="B18" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="60">
         <v>1</v>
       </c>
-      <c r="B19" s="96" t="s">
-        <v>248</v>
-      </c>
-      <c r="C19" s="97"/>
-      <c r="D19" s="97"/>
+      <c r="B19" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2278,973 +2531,973 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC84D6C1-E53B-44EB-A486-CBB464611D59}">
   <dimension ref="A1:G79"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.578125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26.83984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.83984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.68359375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25" style="3" customWidth="1"/>
     <col min="6" max="6" width="34" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.578125" style="3"/>
+    <col min="7" max="7" width="25.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" ht="30">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="75">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="60">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="90">
       <c r="A7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="8" spans="1:7" ht="90">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="60">
       <c r="A9" s="2" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="F9" s="51" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="375">
+      <c r="A10" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="52" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="316.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="52" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="52" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="52" t="s">
-        <v>26</v>
-      </c>
       <c r="E10" s="52" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="F10" s="52" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="231" x14ac:dyDescent="0.55000000000000004">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="247.5">
       <c r="A11" s="5" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="F11" s="45" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="G11" s="5"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:7">
       <c r="C12" s="54"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="73" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="73"/>
-    </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="73"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:7">
+      <c r="A14" s="84" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="84"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="84"/>
+      <c r="E14" s="84"/>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1">
+      <c r="A15" s="84"/>
+      <c r="B15" s="84"/>
+      <c r="C15" s="84"/>
+      <c r="D15" s="84"/>
+      <c r="E15" s="84"/>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" s="6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="84" t="s">
-        <v>71</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="34.5" customHeight="1">
+      <c r="A17" s="95" t="s">
+        <v>94</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="84"/>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="95"/>
       <c r="B18" s="10" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="84"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="95"/>
       <c r="B19" s="10" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="E19" s="8"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="84"/>
+    <row r="20" spans="1:6">
+      <c r="A20" s="95"/>
       <c r="B20" s="10" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="11" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="E20" s="8"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="85"/>
-      <c r="B21" s="85"/>
-      <c r="C21" s="85"/>
-      <c r="D21" s="85"/>
-      <c r="E21" s="85"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="72" t="s">
-        <v>82</v>
+    <row r="21" spans="1:6">
+      <c r="A21" s="96"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="96"/>
+      <c r="D21" s="96"/>
+      <c r="E21" s="96"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="83" t="s">
+        <v>105</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E22" s="86" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="72"/>
+        <v>102</v>
+      </c>
+      <c r="E22" s="97" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="83"/>
       <c r="B23" s="10" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E23" s="86"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="72"/>
+        <v>104</v>
+      </c>
+      <c r="E23" s="97"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="83"/>
       <c r="B24" s="15" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:6">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="72" t="s">
-        <v>88</v>
+    <row r="26" spans="1:6">
+      <c r="A26" s="83" t="s">
+        <v>111</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E26" s="57"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="72"/>
+        <v>102</v>
+      </c>
+      <c r="E26" s="68"/>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="83"/>
       <c r="B27" s="10" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E27" s="57"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="72"/>
+        <v>104</v>
+      </c>
+      <c r="E27" s="68"/>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="83"/>
       <c r="B28" s="15" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
     </row>
-    <row r="30" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="72" t="s">
-        <v>90</v>
+    <row r="30" spans="1:6" ht="15" customHeight="1">
+      <c r="A30" s="83" t="s">
+        <v>113</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="E30" s="83"/>
+        <v>115</v>
+      </c>
+      <c r="E30" s="94"/>
       <c r="F30" s="48" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="72"/>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="83"/>
       <c r="B31" s="19" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E31" s="83"/>
+        <v>102</v>
+      </c>
+      <c r="E31" s="94"/>
       <c r="F31" s="49" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="72"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="83"/>
       <c r="B32" s="20" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E32" s="83"/>
+        <v>104</v>
+      </c>
+      <c r="E32" s="94"/>
       <c r="F32" s="50" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="72"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="83"/>
       <c r="B33" s="20" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="D33" s="11"/>
       <c r="E33" s="44" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="F33" s="49" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="72"/>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="83"/>
       <c r="B34" s="21" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="45" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="F34" s="50" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="72"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="83"/>
       <c r="B35" s="22" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="45" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="F35" s="46"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="72"/>
+    <row r="36" spans="1:6">
+      <c r="A36" s="83"/>
       <c r="B36" s="22" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="45" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="F36" s="46"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="72"/>
+    <row r="37" spans="1:6">
+      <c r="A37" s="83"/>
       <c r="B37" s="22" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="45" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F37" s="46"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="72"/>
+    <row r="38" spans="1:6">
+      <c r="A38" s="83"/>
       <c r="B38" s="22" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="45" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="F38" s="47"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="72" t="s">
-        <v>118</v>
+    <row r="40" spans="1:6">
+      <c r="A40" s="83" t="s">
+        <v>141</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E40" s="57"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="72"/>
+        <v>102</v>
+      </c>
+      <c r="E40" s="68"/>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="83"/>
       <c r="B41" s="10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E41" s="57"/>
-    </row>
-    <row r="42" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="72"/>
+        <v>104</v>
+      </c>
+      <c r="E41" s="68"/>
+    </row>
+    <row r="42" spans="1:6" ht="37.5" customHeight="1">
+      <c r="A42" s="83"/>
       <c r="B42" s="15" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="32" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" s="24"/>
       <c r="B43" s="25"/>
       <c r="C43" s="26"/>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="72" t="s">
-        <v>123</v>
+    <row r="44" spans="1:6">
+      <c r="A44" s="83" t="s">
+        <v>146</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="C44" s="17"/>
       <c r="D44" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E44" s="57"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="72"/>
+        <v>102</v>
+      </c>
+      <c r="E44" s="68"/>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="83"/>
       <c r="B45" s="10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E45" s="57"/>
-    </row>
-    <row r="46" spans="1:6" ht="52.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="72"/>
+        <v>104</v>
+      </c>
+      <c r="E45" s="68"/>
+    </row>
+    <row r="46" spans="1:6" ht="56.25">
+      <c r="A46" s="83"/>
       <c r="B46" s="15" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="32" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47" s="24"/>
       <c r="B47" s="33"/>
       <c r="C47" s="33"/>
       <c r="D47" s="34"/>
       <c r="E47" s="35"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="80" t="s">
-        <v>127</v>
-      </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="81"/>
-      <c r="E48" s="82"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="78" t="s">
-        <v>128</v>
+    <row r="48" spans="1:6">
+      <c r="A48" s="91" t="s">
+        <v>150</v>
+      </c>
+      <c r="B48" s="92"/>
+      <c r="C48" s="92"/>
+      <c r="D48" s="92"/>
+      <c r="E48" s="93"/>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="89" t="s">
+        <v>23</v>
       </c>
       <c r="B49" s="30" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="31" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="E49" s="12"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" s="79"/>
+    <row r="50" spans="1:6">
+      <c r="A50" s="90"/>
       <c r="B50" s="10" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="17"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:6">
       <c r="B51" s="5"/>
       <c r="C51" s="36" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
     </row>
-    <row r="52" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:6" ht="30">
       <c r="B52" s="5"/>
       <c r="C52" s="36" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="58" t="s">
-        <v>135</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="69" t="s">
+        <v>157</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E54" s="57"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="59"/>
+        <v>102</v>
+      </c>
+      <c r="E54" s="68"/>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="70"/>
       <c r="B55" s="10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E55" s="57"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="59"/>
+        <v>104</v>
+      </c>
+      <c r="E55" s="68"/>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="70"/>
       <c r="B56" s="27" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="C56" s="28" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="D56" s="29"/>
       <c r="E56" s="37"/>
     </row>
-    <row r="57" spans="1:6" ht="31.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="60"/>
+    <row r="57" spans="1:6" ht="45">
+      <c r="A57" s="71"/>
       <c r="B57" s="23" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="D57" s="5"/>
       <c r="E57" s="38" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="74" t="s">
-        <v>141</v>
-      </c>
-      <c r="B59" s="74"/>
-      <c r="C59" s="74"/>
-      <c r="D59" s="74"/>
-      <c r="E59" s="75"/>
-      <c r="F59" s="55" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="15" customHeight="1">
+      <c r="A59" s="85" t="s">
+        <v>163</v>
+      </c>
+      <c r="B59" s="85"/>
+      <c r="C59" s="85"/>
+      <c r="D59" s="85"/>
+      <c r="E59" s="86"/>
+      <c r="F59" s="66" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="87"/>
+      <c r="B60" s="87"/>
+      <c r="C60" s="87"/>
+      <c r="D60" s="87"/>
+      <c r="E60" s="88"/>
+      <c r="F60" s="67"/>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="15" customHeight="1">
+      <c r="A62" s="83" t="s">
+        <v>166</v>
+      </c>
+      <c r="B62" s="19" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="76"/>
-      <c r="B60" s="76"/>
-      <c r="C60" s="76"/>
-      <c r="D60" s="76"/>
-      <c r="E60" s="77"/>
-      <c r="F60" s="56"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="B61" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C61" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="B62" s="19" t="s">
-        <v>119</v>
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="E62" s="57"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="72"/>
+        <v>167</v>
+      </c>
+      <c r="E62" s="68"/>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="83"/>
       <c r="B63" s="20" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E63" s="57"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="72"/>
+        <v>104</v>
+      </c>
+      <c r="E63" s="68"/>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="83"/>
       <c r="B64" s="41" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="C64" s="28"/>
       <c r="D64" s="40" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="E64" s="37"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="72"/>
+    <row r="65" spans="1:5">
+      <c r="A65" s="83"/>
       <c r="B65" s="22" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="C65" s="39" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A66" s="72"/>
+    <row r="66" spans="1:5">
+      <c r="A66" s="83"/>
       <c r="B66" s="22" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="C66" s="39" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="72"/>
+    <row r="67" spans="1:5">
+      <c r="A67" s="83"/>
       <c r="B67" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="C67" s="63"/>
-      <c r="D67" s="66"/>
-      <c r="E67" s="69" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A68" s="72"/>
+        <v>171</v>
+      </c>
+      <c r="C67" s="74"/>
+      <c r="D67" s="77"/>
+      <c r="E67" s="80" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="83"/>
       <c r="B68" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="C68" s="64"/>
-      <c r="D68" s="67"/>
-      <c r="E68" s="70"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="72"/>
+        <v>173</v>
+      </c>
+      <c r="C68" s="75"/>
+      <c r="D68" s="78"/>
+      <c r="E68" s="81"/>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="83"/>
       <c r="B69" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="C69" s="65"/>
-      <c r="D69" s="68"/>
-      <c r="E69" s="71"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A71" s="72" t="s">
-        <v>30</v>
+        <v>174</v>
+      </c>
+      <c r="C69" s="76"/>
+      <c r="D69" s="79"/>
+      <c r="E69" s="82"/>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="83" t="s">
+        <v>22</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="11" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="E71" s="17"/>
     </row>
-    <row r="72" spans="1:5" ht="31.5" x14ac:dyDescent="0.4">
-      <c r="A72" s="72"/>
+    <row r="72" spans="1:5" ht="33.75">
+      <c r="A72" s="83"/>
       <c r="B72" s="15" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="C72" s="18" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="43" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="21" x14ac:dyDescent="0.55000000000000004">
-      <c r="A73" s="72"/>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="22.5">
+      <c r="A73" s="83"/>
       <c r="B73" s="23" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="D73" s="5"/>
       <c r="E73" s="32" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A74" s="72"/>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="83"/>
       <c r="B74" s="23" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="38" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
       <c r="A75" s="42"/>
     </row>
-    <row r="76" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A76" s="58" t="s">
-        <v>163</v>
+    <row r="76" spans="1:5" ht="15" customHeight="1">
+      <c r="A76" s="69" t="s">
+        <v>21</v>
       </c>
       <c r="B76" s="16" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="C76" s="17"/>
       <c r="D76" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="E76" s="57"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A77" s="59"/>
+        <v>167</v>
+      </c>
+      <c r="E76" s="68"/>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="70"/>
       <c r="B77" s="10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E77" s="57"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A78" s="59"/>
+        <v>104</v>
+      </c>
+      <c r="E77" s="68"/>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="70"/>
       <c r="B78" s="27" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
       <c r="C78" s="28" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="D78" s="29"/>
-      <c r="E78" s="61" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A79" s="60"/>
+      <c r="E78" s="72" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="23.25" customHeight="1">
+      <c r="A79" s="71"/>
       <c r="B79" s="23" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="D79" s="5"/>
-      <c r="E79" s="62"/>
+      <c r="E79" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="28">
@@ -3284,347 +3537,842 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95D1DD5F-2709-422A-8EBB-A97750EC39C5}">
-  <dimension ref="A1:C31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:J34"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.26171875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.68359375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" style="51" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="51" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="51" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="51" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="51" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="51" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="51" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="1.42578125" style="62" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="51"/>
+    <col min="10" max="10" width="17.5703125" style="51" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="51"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="87" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="63" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="63" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1" s="63" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="63" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" s="63" t="s">
+        <v>195</v>
+      </c>
+      <c r="G1" s="63" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="51" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="51">
+        <v>0</v>
+      </c>
+      <c r="C2" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D2" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" s="51" t="s">
+        <v>200</v>
+      </c>
+      <c r="F2" s="51" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" s="51" t="s">
+        <v>201</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="51" t="s">
+        <v>203</v>
+      </c>
+      <c r="B3" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C3" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D3" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E3" s="51" t="s">
+        <v>204</v>
+      </c>
+      <c r="F3" s="51" t="s">
+        <v>205</v>
+      </c>
+      <c r="G3" s="51" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C4" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" s="51" t="s">
+        <v>209</v>
+      </c>
+      <c r="G4" s="51" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C5" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E5" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="G5" s="51" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="51" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="51">
+        <v>7.5</v>
+      </c>
+      <c r="C6" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D6" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E6" s="51" t="s">
+        <v>216</v>
+      </c>
+      <c r="F6" s="51" t="s">
+        <v>217</v>
+      </c>
+      <c r="G6" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H6" s="51" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="51" t="s">
+        <v>220</v>
+      </c>
+      <c r="B7" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C7" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D7" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E7" s="51" t="s">
+        <v>222</v>
+      </c>
+      <c r="F7" s="64" t="s">
+        <v>223</v>
+      </c>
+      <c r="G7" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="51" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" s="51">
+        <v>5</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="51" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15" customHeight="1">
+      <c r="A9" s="51" t="s">
+        <v>228</v>
+      </c>
+      <c r="B9" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="51" t="s">
+        <v>229</v>
+      </c>
+      <c r="F9" s="51" t="s">
+        <v>230</v>
+      </c>
+      <c r="G9" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="B10" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C10" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E10" s="51" t="s">
+        <v>232</v>
+      </c>
+      <c r="F10" s="51" t="s">
+        <v>233</v>
+      </c>
+      <c r="G10" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="51" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11" s="51" t="s">
+        <v>122</v>
+      </c>
+      <c r="G11" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="51" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C12" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D12" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E12" s="51" t="s">
+        <v>237</v>
+      </c>
+      <c r="F12" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="G12" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="51" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C13" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>239</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>240</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="51" t="s">
+        <v>241</v>
+      </c>
+      <c r="B14" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C14" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D14" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E14" s="51" t="s">
+        <v>242</v>
+      </c>
+      <c r="F14" s="51" t="s">
+        <v>243</v>
+      </c>
+      <c r="G14" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="51" t="s">
+        <v>244</v>
+      </c>
+      <c r="B15" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C15" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>245</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C16" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>247</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>248</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="51" t="s">
+        <v>225</v>
+      </c>
+      <c r="B17" s="51">
+        <v>5</v>
+      </c>
+      <c r="C17" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D17" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" s="51" t="s">
+        <v>250</v>
+      </c>
+      <c r="F17" s="51" t="s">
+        <v>251</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="51">
+        <v>5</v>
+      </c>
+      <c r="C18" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D18" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E18" s="51" t="s">
+        <v>252</v>
+      </c>
+      <c r="F18" s="51" t="s">
+        <v>126</v>
+      </c>
+      <c r="G18" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="51">
+        <v>5</v>
+      </c>
+      <c r="C19" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E19" s="51" t="s">
+        <v>253</v>
+      </c>
+      <c r="F19" s="51" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" s="51">
+        <v>5</v>
+      </c>
+      <c r="C20" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E20" s="51" t="s">
+        <v>254</v>
+      </c>
+      <c r="F20" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="G20" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B21" s="51">
+        <v>5</v>
+      </c>
+      <c r="C21" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>255</v>
+      </c>
+      <c r="F21" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="51" t="s">
+        <v>256</v>
+      </c>
+      <c r="B22" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C22" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22" s="51" t="s">
+        <v>257</v>
+      </c>
+      <c r="E22" s="51" t="s">
+        <v>258</v>
+      </c>
+      <c r="F22" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="G22" s="51" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="51" t="s">
+        <v>256</v>
+      </c>
+      <c r="B23" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C23" s="51" t="s">
+        <v>260</v>
+      </c>
+      <c r="D23" s="51" t="s">
+        <v>257</v>
+      </c>
+      <c r="E23" s="51" t="s">
+        <v>261</v>
+      </c>
+      <c r="F23" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="G23" s="51" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="51" t="s">
+        <v>263</v>
+      </c>
+      <c r="B24" s="51">
+        <v>5</v>
+      </c>
+      <c r="C24" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D24" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E24" s="51" t="s">
+        <v>265</v>
+      </c>
+      <c r="F24" s="51" t="s">
+        <v>266</v>
+      </c>
+      <c r="G24" s="51" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="51" t="s">
+        <v>263</v>
+      </c>
+      <c r="B25" s="51">
+        <v>5</v>
+      </c>
+      <c r="C25" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E25" s="51" t="s">
+        <v>268</v>
+      </c>
+      <c r="F25" s="51" t="s">
+        <v>269</v>
+      </c>
+      <c r="G25" s="51" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="51" t="s">
+        <v>271</v>
+      </c>
+      <c r="B26" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C26" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E26" s="51" t="s">
+        <v>272</v>
+      </c>
+      <c r="F26" s="51" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="51" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15" customHeight="1">
+      <c r="A27" s="51" t="s">
+        <v>274</v>
+      </c>
+      <c r="B27" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C27" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E27" s="51" t="s">
+        <v>275</v>
+      </c>
+      <c r="F27" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="51" t="s">
+        <v>277</v>
+      </c>
+      <c r="B28" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C28" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E28" s="51" t="s">
+        <v>278</v>
+      </c>
+      <c r="F28" s="51" t="s">
         <v>169</v>
       </c>
-      <c r="B1" s="87" t="s">
-        <v>170</v>
-      </c>
-      <c r="C1" s="87" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="88" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="51" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="88"/>
-      <c r="B3" s="51" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="51" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="51" t="s">
-        <v>174</v>
-      </c>
-      <c r="B4" s="51" t="s">
-        <v>175</v>
-      </c>
-      <c r="C4" s="51" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="51" t="s">
-        <v>177</v>
-      </c>
-      <c r="B5" s="51" t="s">
-        <v>178</v>
-      </c>
-      <c r="C5" s="51" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B6" s="51" t="s">
-        <v>180</v>
-      </c>
-      <c r="C6" s="51" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="51" t="s">
-        <v>181</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>182</v>
-      </c>
-      <c r="C7" s="51" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="51" t="s">
-        <v>184</v>
-      </c>
-      <c r="B8" s="51" t="s">
-        <v>137</v>
-      </c>
-      <c r="C8" s="51" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="89" t="s">
-        <v>90</v>
-      </c>
-      <c r="B9" s="51" t="s">
-        <v>99</v>
-      </c>
-      <c r="C9" s="51" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="89"/>
-      <c r="B10" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" s="51" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="89"/>
-      <c r="B11" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" s="51" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="89"/>
-      <c r="B12" s="51" t="s">
-        <v>110</v>
-      </c>
-      <c r="C12" s="51" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="89"/>
-      <c r="B13" s="51" t="s">
+      <c r="G28" s="51" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="51" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="89"/>
-      <c r="B14" s="51" t="s">
-        <v>116</v>
-      </c>
-      <c r="C14" s="51" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="51" t="s">
-        <v>192</v>
-      </c>
-      <c r="B15" s="51" t="s">
-        <v>193</v>
-      </c>
-      <c r="C15" s="51" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="B16" s="51" t="s">
-        <v>196</v>
-      </c>
-      <c r="C16" s="51" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="51" t="s">
+      <c r="B29" s="51">
+        <v>5</v>
+      </c>
+      <c r="C29" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E29" s="51" t="s">
+        <v>280</v>
+      </c>
+      <c r="F29" s="51" t="s">
+        <v>281</v>
+      </c>
+      <c r="G29" s="51" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15" customHeight="1">
+      <c r="A30" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="51">
+        <v>5</v>
+      </c>
+      <c r="C30" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E30" s="98" t="s">
+        <v>283</v>
+      </c>
+      <c r="F30" s="98" t="s">
+        <v>284</v>
+      </c>
+      <c r="G30" s="51" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="51" t="s">
+        <v>286</v>
+      </c>
+      <c r="B31" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C31" s="51" t="s">
         <v>198</v>
       </c>
-      <c r="B17" s="51" t="s">
-        <v>199</v>
-      </c>
-      <c r="C17" s="51" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="51" t="s">
-        <v>201</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>202</v>
-      </c>
-      <c r="C18" s="51" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>205</v>
-      </c>
-      <c r="C19" s="51" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="51" t="s">
-        <v>207</v>
-      </c>
-      <c r="B20" s="51" t="s">
-        <v>208</v>
-      </c>
-      <c r="C20" s="51" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="51" t="s">
-        <v>210</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>211</v>
-      </c>
-      <c r="C21" s="51" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="51" t="s">
-        <v>128</v>
-      </c>
-      <c r="B22" s="51" t="s">
-        <v>213</v>
-      </c>
-      <c r="C22" s="51" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="88" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="51" t="s">
-        <v>137</v>
-      </c>
-      <c r="C23" s="51" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="88"/>
-      <c r="B24" s="51" t="s">
-        <v>139</v>
-      </c>
-      <c r="C24" s="51" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="88" t="s">
-        <v>217</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>147</v>
-      </c>
-      <c r="C25" s="51" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="88"/>
-      <c r="B26" s="51" t="s">
-        <v>148</v>
-      </c>
-      <c r="C26" s="51" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="89" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="51" t="s">
-        <v>220</v>
-      </c>
-      <c r="C27" s="51" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="89"/>
-      <c r="B28" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="C28" s="51" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="89"/>
-      <c r="B29" s="51" t="s">
-        <v>224</v>
-      </c>
-      <c r="C29" s="51" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="89" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="51" t="s">
-        <v>165</v>
-      </c>
-      <c r="C30" s="51" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="89"/>
-      <c r="B31" s="51" t="s">
-        <v>168</v>
-      </c>
-      <c r="C31" s="51" t="s">
-        <v>227</v>
+      <c r="D31" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="E31" s="98" t="s">
+        <v>288</v>
+      </c>
+      <c r="F31" s="98" t="s">
+        <v>161</v>
+      </c>
+      <c r="G31" s="51" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="51" t="s">
+        <v>286</v>
+      </c>
+      <c r="B32" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C32" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="E32" s="98" t="s">
+        <v>290</v>
+      </c>
+      <c r="F32" s="98" t="s">
+        <v>159</v>
+      </c>
+      <c r="G32" s="51" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="51" t="s">
+        <v>292</v>
+      </c>
+      <c r="B33" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C33" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="E33" s="98" t="s">
+        <v>293</v>
+      </c>
+      <c r="F33" s="98" t="s">
+        <v>294</v>
+      </c>
+      <c r="G33" s="51" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="51" t="s">
+        <v>292</v>
+      </c>
+      <c r="B34" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="C34" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="E34" s="51" t="s">
+        <v>296</v>
+      </c>
+      <c r="F34" s="51" t="s">
+        <v>297</v>
+      </c>
+      <c r="G34" s="51" t="s">
+        <v>298</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A30:A31"/>
-  </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="d2a0b54d-44c5-4b89-a4c6-11e478ac2bb7" xsi:nil="true"/>
@@ -3632,7 +4380,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AABD4A0AF4D47242A1863BD8A28AFF99" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9fd1c8938e90e57e83ed08a21189a5a5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d2a0b54d-44c5-4b89-a4c6-11e478ac2bb7" xmlns:ns4="5ede1437-6869-4495-baa0-a24edee2ad6a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="37eac2a113e6f746f5f658fa36d4e3bc" ns3:_="" ns4:_="">
     <xsd:import namespace="d2a0b54d-44c5-4b89-a4c6-11e478ac2bb7"/>
@@ -3885,55 +4633,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6DE7DE9-56EF-447D-9504-04CC9F9A75DD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="5ede1437-6869-4495-baa0-a24edee2ad6a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="d2a0b54d-44c5-4b89-a4c6-11e478ac2bb7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79518780-8CB7-4055-9EE6-E8513603408F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C5CEDEC-202B-43F2-B1C0-4261D400BE7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d2a0b54d-44c5-4b89-a4c6-11e478ac2bb7"/>
-    <ds:schemaRef ds:uri="5ede1437-6869-4495-baa0-a24edee2ad6a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6DE7DE9-56EF-447D-9504-04CC9F9A75DD}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79518780-8CB7-4055-9EE6-E8513603408F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C5CEDEC-202B-43F2-B1C0-4261D400BE7B}"/>
 </file>
</xml_diff>